<commit_message>
Fix renamed audio and rhythm codes
</commit_message>
<xml_diff>
--- a/docs/tabulka-hnev.xlsx
+++ b/docs/tabulka-hnev.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Kajik BP web\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Kajik BP web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CC9BD7C-900D-4CFC-8F13-C07042DF0E86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66008CA0-BB33-499C-B510-E6E268027F8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{8585123D-28A0-4BD2-87B7-9BF3FF211F10}"/>
+    <workbookView xWindow="-18720" yWindow="3765" windowWidth="21600" windowHeight="11385" xr2:uid="{8585123D-28A0-4BD2-87B7-9BF3FF211F10}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -701,7 +701,7 @@
   <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" customWidth="1"/>
+    <col min="1" max="1" width="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>